<commit_message>
fixed another mistake in the excel, updated the data, updated the library.
</commit_message>
<xml_diff>
--- a/uploads/labs_spring.xlsx
+++ b/uploads/labs_spring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/DimiTrianta/Desktop/ds_dynamic_schedule/uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E07537DB-BC1D-1245-B167-26323EFE0D1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{2956A16A-84A5-294F-A9D3-29069DC365E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{12B5CF23-F2A4-A143-A910-D3B11DBC6ACE}"/>
   </bookViews>
@@ -23,15 +23,6 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -138,9 +129,6 @@
     <t>ΑΝΑΛΥΣΗ ΔΕΔΟΜΕΝΩΝ</t>
   </si>
   <si>
-    <t>AΣΥΡΜΑΤΕΣ ΕΠΙΚΟΙΝΩΝΙΕΣ</t>
-  </si>
-  <si>
     <t>ΠΡΩΤΟΚΟΛΛΑ ΔΙΑΔΙΚΤΥΟΥ</t>
   </si>
   <si>
@@ -251,6 +239,9 @@
   </si>
   <si>
     <t>ΚΟΙΝΩΝΙΚΑ ΔΙΚΤΥΑ</t>
+  </si>
+  <si>
+    <t>ΑΣΥΡΜΑΤΕΣ ΕΠΙΚΟΙΝΩΝΙΕΣ</t>
   </si>
 </sst>
 </file>
@@ -613,7 +604,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -621,22 +612,22 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -648,8 +639,8 @@
     <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -675,10 +666,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -697,7 +685,7 @@
     <xf numFmtId="49" fontId="18" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="19" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -709,9 +697,6 @@
     <xf numFmtId="49" fontId="14" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="26" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -720,9 +705,6 @@
     </xf>
     <xf numFmtId="0" fontId="26" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="19" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -751,7 +733,7 @@
     <xf numFmtId="49" fontId="14" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="16" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -776,6 +758,75 @@
     <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="5" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="14" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -785,160 +836,91 @@
     <xf numFmtId="49" fontId="14" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="5" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="5" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="5" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="5" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="5" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="5" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="5" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="16" fillId="5" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="5" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="5" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1262,50 +1244,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="84" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="104"/>
-      <c r="C1" s="104"/>
-      <c r="D1" s="104"/>
-      <c r="E1" s="104"/>
-      <c r="F1" s="104"/>
-      <c r="G1" s="104"/>
+      <c r="B1" s="84"/>
+      <c r="C1" s="84"/>
+      <c r="D1" s="84"/>
+      <c r="E1" s="84"/>
+      <c r="F1" s="84"/>
+      <c r="G1" s="84"/>
     </row>
     <row r="2" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="104" t="s">
+      <c r="A2" s="84" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="104"/>
-      <c r="C2" s="104"/>
-      <c r="D2" s="104"/>
-      <c r="E2" s="104"/>
-      <c r="F2" s="104"/>
-      <c r="G2" s="104"/>
+      <c r="B2" s="84"/>
+      <c r="C2" s="84"/>
+      <c r="D2" s="84"/>
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="84"/>
       <c r="H2" s="3"/>
     </row>
     <row r="3" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="104" t="s">
+      <c r="A3" s="84" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="104"/>
-      <c r="C3" s="104"/>
-      <c r="D3" s="104"/>
-      <c r="E3" s="104"/>
-      <c r="F3" s="104"/>
-      <c r="G3" s="104"/>
+      <c r="B3" s="84"/>
+      <c r="C3" s="84"/>
+      <c r="D3" s="84"/>
+      <c r="E3" s="84"/>
+      <c r="F3" s="84"/>
+      <c r="G3" s="84"/>
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="104" t="s">
-        <v>60</v>
-      </c>
-      <c r="B4" s="104"/>
-      <c r="C4" s="104"/>
-      <c r="D4" s="104"/>
-      <c r="E4" s="104"/>
-      <c r="F4" s="104"/>
-      <c r="G4" s="104"/>
+      <c r="A4" s="84" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="84"/>
+      <c r="C4" s="84"/>
+      <c r="D4" s="84"/>
+      <c r="E4" s="84"/>
+      <c r="F4" s="84"/>
+      <c r="G4" s="84"/>
       <c r="H4" s="8"/>
     </row>
     <row r="5" spans="1:9" ht="22" x14ac:dyDescent="0.15">
@@ -1333,7 +1315,7 @@
       <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="32" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="12"/>
@@ -1348,10 +1330,10 @@
         <v>11</v>
       </c>
       <c r="B7" s="15"/>
-      <c r="C7" s="68" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="44"/>
+      <c r="C7" s="56" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="41"/>
       <c r="E7" s="16"/>
       <c r="F7" s="17"/>
       <c r="G7" s="18" t="s">
@@ -1362,18 +1344,18 @@
       <c r="A8" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="105" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" s="69"/>
-      <c r="D8" s="106" t="s">
-        <v>69</v>
-      </c>
-      <c r="E8" s="68" t="s">
-        <v>64</v>
-      </c>
-      <c r="F8" s="77" t="s">
-        <v>67</v>
+      <c r="B8" s="85" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="57"/>
+      <c r="D8" s="81" t="s">
+        <v>68</v>
+      </c>
+      <c r="E8" s="56" t="s">
+        <v>63</v>
+      </c>
+      <c r="F8" s="71" t="s">
+        <v>66</v>
       </c>
       <c r="G8" s="19" t="s">
         <v>15</v>
@@ -1383,13 +1365,13 @@
       <c r="A9" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="105"/>
-      <c r="C9" s="68" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="107"/>
-      <c r="E9" s="69"/>
-      <c r="F9" s="78"/>
+      <c r="B9" s="85"/>
+      <c r="C9" s="56" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="82"/>
+      <c r="E9" s="57"/>
+      <c r="F9" s="72"/>
       <c r="G9" s="20" t="s">
         <v>16</v>
       </c>
@@ -1399,17 +1381,17 @@
       <c r="A10" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="68" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="69"/>
-      <c r="D10" s="83" t="s">
+      <c r="B10" s="56" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="57"/>
+      <c r="D10" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="68" t="s">
-        <v>64</v>
-      </c>
-      <c r="F10" s="54"/>
+      <c r="E10" s="56" t="s">
+        <v>63</v>
+      </c>
+      <c r="F10" s="51"/>
       <c r="G10" s="21" t="s">
         <v>17</v>
       </c>
@@ -1418,11 +1400,11 @@
       <c r="A11" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="69"/>
+      <c r="B11" s="57"/>
       <c r="C11" s="15"/>
-      <c r="D11" s="84"/>
-      <c r="E11" s="69"/>
-      <c r="F11" s="65" t="s">
+      <c r="D11" s="74"/>
+      <c r="E11" s="57"/>
+      <c r="F11" s="77" t="s">
         <v>9</v>
       </c>
       <c r="G11" s="12"/>
@@ -1431,17 +1413,17 @@
       <c r="A12" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="68" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" s="65" t="s">
+      <c r="B12" s="56" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="D12" s="83" t="s">
+      <c r="D12" s="73" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="41"/>
-      <c r="F12" s="65"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="77"/>
       <c r="G12" s="12"/>
       <c r="H12" s="2"/>
     </row>
@@ -1449,74 +1431,74 @@
       <c r="A13" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="69"/>
-      <c r="C13" s="65"/>
-      <c r="D13" s="84"/>
-      <c r="E13" s="85" t="s">
-        <v>55</v>
-      </c>
-      <c r="F13" s="65" t="s">
+      <c r="B13" s="57"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="74"/>
+      <c r="E13" s="94" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="G13" s="87"/>
+      <c r="G13" s="91"/>
     </row>
     <row r="14" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="76" t="s">
-        <v>59</v>
-      </c>
-      <c r="C14" s="65" t="s">
+      <c r="B14" s="58" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="D14" s="83" t="s">
-        <v>48</v>
-      </c>
-      <c r="E14" s="86"/>
-      <c r="F14" s="65"/>
-      <c r="G14" s="88"/>
-      <c r="H14" s="97"/>
+      <c r="D14" s="73" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" s="95"/>
+      <c r="F14" s="77"/>
+      <c r="G14" s="92"/>
+      <c r="H14" s="99"/>
     </row>
     <row r="15" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="76"/>
-      <c r="C15" s="65"/>
-      <c r="D15" s="84"/>
-      <c r="E15" s="83" t="s">
+      <c r="B15" s="58"/>
+      <c r="C15" s="77"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="73" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="74" t="s">
-        <v>46</v>
-      </c>
-      <c r="G15" s="88"/>
-      <c r="H15" s="97"/>
-      <c r="I15" s="99"/>
+      <c r="F15" s="60" t="s">
+        <v>45</v>
+      </c>
+      <c r="G15" s="92"/>
+      <c r="H15" s="99"/>
+      <c r="I15" s="86"/>
     </row>
     <row r="16" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="50"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="84"/>
-      <c r="F16" s="75"/>
-      <c r="G16" s="88"/>
-      <c r="I16" s="99"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="61"/>
+      <c r="G16" s="92"/>
+      <c r="I16" s="86"/>
     </row>
     <row r="17" spans="1:11" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="34" t="s">
+      <c r="A17" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="24"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="88"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="92"/>
     </row>
     <row r="18" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="14" t="s">
@@ -1525,218 +1507,218 @@
       <c r="B18" s="22"/>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="88"/>
-      <c r="I18" s="101"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="92"/>
+      <c r="I18" s="88"/>
     </row>
     <row r="19" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="68" t="s">
+      <c r="B19" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="65" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="102" t="s">
-        <v>40</v>
-      </c>
-      <c r="E19" s="76" t="s">
-        <v>59</v>
-      </c>
-      <c r="F19" s="82" t="s">
+      <c r="C19" s="77" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" s="89" t="s">
+        <v>39</v>
+      </c>
+      <c r="E19" s="58" t="s">
         <v>58</v>
       </c>
-      <c r="G19" s="88"/>
+      <c r="F19" s="75" t="s">
+        <v>57</v>
+      </c>
+      <c r="G19" s="92"/>
       <c r="H19" s="6"/>
-      <c r="I19" s="101"/>
+      <c r="I19" s="88"/>
     </row>
     <row r="20" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="69"/>
-      <c r="C20" s="65"/>
-      <c r="D20" s="103"/>
-      <c r="E20" s="76"/>
-      <c r="F20" s="69"/>
-      <c r="G20" s="88"/>
-      <c r="I20" s="101"/>
+      <c r="B20" s="57"/>
+      <c r="C20" s="77"/>
+      <c r="D20" s="90"/>
+      <c r="E20" s="58"/>
+      <c r="F20" s="57"/>
+      <c r="G20" s="92"/>
+      <c r="I20" s="88"/>
     </row>
     <row r="21" spans="1:11" ht="36.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="68" t="s">
-        <v>37</v>
-      </c>
-      <c r="C21" s="61" t="s">
-        <v>33</v>
-      </c>
-      <c r="D21" s="83" t="s">
-        <v>48</v>
-      </c>
-      <c r="E21" s="76" t="s">
-        <v>59</v>
-      </c>
-      <c r="F21" s="96"/>
-      <c r="G21" s="88"/>
-      <c r="I21" s="101"/>
+      <c r="B21" s="56" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="59" t="s">
+        <v>70</v>
+      </c>
+      <c r="D21" s="73" t="s">
+        <v>47</v>
+      </c>
+      <c r="E21" s="58" t="s">
+        <v>58</v>
+      </c>
+      <c r="F21" s="98"/>
+      <c r="G21" s="92"/>
+      <c r="I21" s="88"/>
     </row>
     <row r="22" spans="1:11" ht="35.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="69"/>
-      <c r="C22" s="61"/>
-      <c r="D22" s="84"/>
-      <c r="E22" s="76"/>
-      <c r="F22" s="96"/>
-      <c r="G22" s="88"/>
+      <c r="B22" s="57"/>
+      <c r="C22" s="59"/>
+      <c r="D22" s="74"/>
+      <c r="E22" s="58"/>
+      <c r="F22" s="98"/>
+      <c r="G22" s="92"/>
     </row>
     <row r="23" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="68" t="s">
+      <c r="B23" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="66" t="s">
-        <v>36</v>
-      </c>
-      <c r="D23" s="83" t="s">
+      <c r="C23" s="106" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="E23" s="25"/>
-      <c r="F23" s="41"/>
-      <c r="G23" s="88"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="38"/>
+      <c r="G23" s="92"/>
     </row>
     <row r="24" spans="1:11" ht="36.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B24" s="69"/>
-      <c r="C24" s="67"/>
-      <c r="D24" s="84"/>
-      <c r="E24" s="83" t="s">
+      <c r="B24" s="57"/>
+      <c r="C24" s="107"/>
+      <c r="D24" s="74"/>
+      <c r="E24" s="73" t="s">
         <v>32</v>
       </c>
-      <c r="F24" s="111" t="s">
-        <v>47</v>
-      </c>
-      <c r="G24" s="88"/>
+      <c r="F24" s="62" t="s">
+        <v>46</v>
+      </c>
+      <c r="G24" s="92"/>
     </row>
     <row r="25" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="B25" s="98" t="s">
-        <v>68</v>
-      </c>
-      <c r="C25" s="73" t="s">
-        <v>36</v>
-      </c>
-      <c r="D25" s="83" t="s">
+      <c r="B25" s="69" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25" s="109" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" s="73" t="s">
         <v>32</v>
       </c>
-      <c r="E25" s="84"/>
-      <c r="F25" s="111"/>
-      <c r="G25" s="88"/>
+      <c r="E25" s="74"/>
+      <c r="F25" s="62"/>
+      <c r="G25" s="92"/>
       <c r="H25" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="41.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="28" t="s">
+      <c r="A26" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="81"/>
-      <c r="C26" s="67"/>
-      <c r="D26" s="84"/>
-      <c r="E26" s="85" t="s">
-        <v>55</v>
-      </c>
-      <c r="F26" s="74" t="s">
+      <c r="B26" s="70"/>
+      <c r="C26" s="107"/>
+      <c r="D26" s="74"/>
+      <c r="E26" s="94" t="s">
         <v>54</v>
       </c>
-      <c r="G26" s="88"/>
+      <c r="F26" s="60" t="s">
+        <v>53</v>
+      </c>
+      <c r="G26" s="92"/>
     </row>
     <row r="27" spans="1:11" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="46"/>
-      <c r="C27" s="49"/>
-      <c r="D27" s="83"/>
-      <c r="E27" s="86"/>
-      <c r="F27" s="75"/>
-      <c r="G27" s="88"/>
+      <c r="B27" s="43"/>
+      <c r="C27" s="46"/>
+      <c r="D27" s="73"/>
+      <c r="E27" s="95"/>
+      <c r="F27" s="61"/>
+      <c r="G27" s="92"/>
     </row>
     <row r="28" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A28" s="39" t="s">
-        <v>50</v>
-      </c>
-      <c r="B28" s="36"/>
-      <c r="C28" s="35"/>
-      <c r="D28" s="84"/>
-      <c r="E28" s="45"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="88"/>
+      <c r="A28" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28" s="34"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="74"/>
+      <c r="E28" s="42"/>
+      <c r="F28" s="35"/>
+      <c r="G28" s="92"/>
     </row>
     <row r="29" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="34" t="s">
+      <c r="A29" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="24"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
+      <c r="B29" s="23"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
       <c r="E29" s="17"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="88"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="92"/>
     </row>
     <row r="30" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B30" s="29"/>
-      <c r="C30" s="40"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="47"/>
-      <c r="F30" s="57"/>
-      <c r="G30" s="88"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="37"/>
+      <c r="D30" s="31"/>
+      <c r="E30" s="44"/>
+      <c r="F30" s="54"/>
+      <c r="G30" s="92"/>
       <c r="H30" s="7"/>
     </row>
     <row r="31" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B31" s="77" t="s">
-        <v>70</v>
-      </c>
-      <c r="C31" s="70" t="s">
-        <v>39</v>
-      </c>
-      <c r="D31" s="77" t="s">
-        <v>52</v>
-      </c>
-      <c r="E31" s="74"/>
-      <c r="F31" s="70"/>
-      <c r="G31" s="88"/>
+      <c r="B31" s="71" t="s">
+        <v>69</v>
+      </c>
+      <c r="C31" s="101" t="s">
+        <v>38</v>
+      </c>
+      <c r="D31" s="71" t="s">
+        <v>51</v>
+      </c>
+      <c r="E31" s="60"/>
+      <c r="F31" s="101"/>
+      <c r="G31" s="92"/>
     </row>
     <row r="32" spans="1:11" ht="36.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B32" s="78"/>
-      <c r="C32" s="71"/>
-      <c r="D32" s="78"/>
-      <c r="E32" s="75"/>
-      <c r="F32" s="72"/>
-      <c r="G32" s="88"/>
-      <c r="H32" s="100"/>
-      <c r="K32" s="95" t="s">
+      <c r="B32" s="72"/>
+      <c r="C32" s="108"/>
+      <c r="D32" s="72"/>
+      <c r="E32" s="61"/>
+      <c r="F32" s="102"/>
+      <c r="G32" s="92"/>
+      <c r="H32" s="87"/>
+      <c r="K32" s="97" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1744,275 +1726,343 @@
       <c r="A33" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B33" s="61"/>
-      <c r="C33" s="72"/>
-      <c r="D33" s="82" t="s">
-        <v>61</v>
-      </c>
-      <c r="E33" s="79" t="s">
-        <v>43</v>
-      </c>
-      <c r="F33" s="42"/>
-      <c r="G33" s="88"/>
-      <c r="H33" s="100"/>
-      <c r="K33" s="95"/>
+      <c r="B33" s="59"/>
+      <c r="C33" s="102"/>
+      <c r="D33" s="75" t="s">
+        <v>60</v>
+      </c>
+      <c r="E33" s="63" t="s">
+        <v>42</v>
+      </c>
+      <c r="F33" s="39"/>
+      <c r="G33" s="92"/>
+      <c r="H33" s="87"/>
+      <c r="K33" s="97"/>
     </row>
     <row r="34" spans="1:11" ht="47.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B34" s="61"/>
-      <c r="C34" s="61"/>
-      <c r="D34" s="108"/>
-      <c r="E34" s="80"/>
-      <c r="F34" s="42"/>
-      <c r="G34" s="88"/>
+      <c r="B34" s="59"/>
+      <c r="C34" s="59"/>
+      <c r="D34" s="76"/>
+      <c r="E34" s="100"/>
+      <c r="F34" s="39"/>
+      <c r="G34" s="92"/>
     </row>
     <row r="35" spans="1:11" ht="34.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B35" s="79"/>
-      <c r="C35" s="61"/>
+      <c r="B35" s="63"/>
+      <c r="C35" s="59"/>
       <c r="D35" s="17"/>
-      <c r="E35" s="81"/>
-      <c r="F35" s="42"/>
-      <c r="G35" s="88"/>
+      <c r="E35" s="70"/>
+      <c r="F35" s="39"/>
+      <c r="G35" s="92"/>
     </row>
     <row r="36" spans="1:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B36" s="110"/>
-      <c r="C36" s="90" t="s">
-        <v>65</v>
-      </c>
-      <c r="D36" s="77" t="s">
-        <v>65</v>
-      </c>
-      <c r="E36" s="98" t="s">
-        <v>53</v>
-      </c>
-      <c r="F36" s="77" t="s">
-        <v>63</v>
-      </c>
-      <c r="G36" s="88"/>
+      <c r="B36" s="65"/>
+      <c r="C36" s="55" t="s">
+        <v>64</v>
+      </c>
+      <c r="D36" s="71" t="s">
+        <v>64</v>
+      </c>
+      <c r="E36" s="69" t="s">
+        <v>52</v>
+      </c>
+      <c r="F36" s="71" t="s">
+        <v>62</v>
+      </c>
+      <c r="G36" s="92"/>
       <c r="H36" s="5"/>
     </row>
     <row r="37" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="B37" s="61" t="s">
-        <v>66</v>
-      </c>
-      <c r="C37" s="90"/>
-      <c r="D37" s="78"/>
-      <c r="E37" s="81"/>
-      <c r="F37" s="78"/>
-      <c r="G37" s="88"/>
+      <c r="B37" s="59" t="s">
+        <v>65</v>
+      </c>
+      <c r="C37" s="55"/>
+      <c r="D37" s="72"/>
+      <c r="E37" s="70"/>
+      <c r="F37" s="72"/>
+      <c r="G37" s="92"/>
       <c r="H37" s="6"/>
     </row>
     <row r="38" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B38" s="61"/>
-      <c r="C38" s="90"/>
-      <c r="D38" s="77" t="s">
-        <v>44</v>
-      </c>
-      <c r="E38" s="74"/>
-      <c r="F38" s="56"/>
-      <c r="G38" s="88"/>
+      <c r="B38" s="59"/>
+      <c r="C38" s="55"/>
+      <c r="D38" s="71" t="s">
+        <v>43</v>
+      </c>
+      <c r="E38" s="60"/>
+      <c r="F38" s="53"/>
+      <c r="G38" s="92"/>
       <c r="H38" s="6"/>
     </row>
     <row r="39" spans="1:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="B39" s="45"/>
-      <c r="C39" s="53"/>
-      <c r="D39" s="78"/>
-      <c r="E39" s="75"/>
-      <c r="F39" s="55"/>
-      <c r="G39" s="88"/>
+      <c r="B39" s="42"/>
+      <c r="C39" s="50"/>
+      <c r="D39" s="72"/>
+      <c r="E39" s="61"/>
+      <c r="F39" s="52"/>
+      <c r="G39" s="92"/>
     </row>
     <row r="40" spans="1:11" ht="23.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A40" s="31"/>
-      <c r="B40" s="23"/>
-      <c r="C40" s="23"/>
-      <c r="D40" s="23"/>
-      <c r="E40" s="23"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="88"/>
+      <c r="A40" s="30"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="92"/>
     </row>
     <row r="41" spans="1:11" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="B41" s="24"/>
-      <c r="C41" s="23"/>
-      <c r="D41" s="23"/>
-      <c r="E41" s="23"/>
-      <c r="F41" s="23"/>
-      <c r="G41" s="88"/>
+      <c r="A41" s="33" t="s">
+        <v>37</v>
+      </c>
+      <c r="B41" s="23"/>
+      <c r="C41" s="14"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="14"/>
+      <c r="G41" s="92"/>
     </row>
     <row r="42" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B42" s="62" t="s">
-        <v>61</v>
-      </c>
-      <c r="C42" s="51"/>
-      <c r="D42" s="94" t="s">
-        <v>45</v>
-      </c>
-      <c r="E42" s="30"/>
-      <c r="F42" s="42"/>
-      <c r="G42" s="88"/>
+      <c r="B42" s="103" t="s">
+        <v>60</v>
+      </c>
+      <c r="C42" s="48"/>
+      <c r="D42" s="96" t="s">
+        <v>44</v>
+      </c>
+      <c r="E42" s="29"/>
+      <c r="F42" s="39"/>
+      <c r="G42" s="92"/>
     </row>
     <row r="43" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B43" s="63"/>
-      <c r="C43" s="74" t="s">
-        <v>42</v>
-      </c>
-      <c r="D43" s="94"/>
-      <c r="E43" s="108" t="s">
-        <v>51</v>
-      </c>
-      <c r="F43" s="74" t="s">
-        <v>62</v>
-      </c>
-      <c r="G43" s="88"/>
+      <c r="B43" s="104"/>
+      <c r="C43" s="60" t="s">
+        <v>41</v>
+      </c>
+      <c r="D43" s="96"/>
+      <c r="E43" s="76" t="s">
+        <v>50</v>
+      </c>
+      <c r="F43" s="60" t="s">
+        <v>61</v>
+      </c>
+      <c r="G43" s="92"/>
     </row>
     <row r="44" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B44" s="64"/>
-      <c r="C44" s="75"/>
-      <c r="D44" s="94"/>
-      <c r="E44" s="109"/>
-      <c r="F44" s="75"/>
-      <c r="G44" s="88"/>
+      <c r="B44" s="105"/>
+      <c r="C44" s="61"/>
+      <c r="D44" s="96"/>
+      <c r="E44" s="83"/>
+      <c r="F44" s="61"/>
+      <c r="G44" s="92"/>
     </row>
     <row r="45" spans="1:11" ht="23.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B45" s="79" t="s">
-        <v>57</v>
-      </c>
-      <c r="C45" s="52"/>
-      <c r="D45" s="91" t="s">
-        <v>47</v>
-      </c>
-      <c r="E45" s="58" t="s">
+      <c r="B45" s="63" t="s">
         <v>56</v>
       </c>
-      <c r="F45" s="90" t="s">
-        <v>49</v>
-      </c>
-      <c r="G45" s="88"/>
+      <c r="C45" s="49"/>
+      <c r="D45" s="66" t="s">
+        <v>46</v>
+      </c>
+      <c r="E45" s="78" t="s">
+        <v>55</v>
+      </c>
+      <c r="F45" s="55" t="s">
+        <v>48</v>
+      </c>
+      <c r="G45" s="92"/>
     </row>
     <row r="46" spans="1:11" ht="39.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B46" s="112"/>
-      <c r="C46" s="61" t="s">
-        <v>66</v>
-      </c>
-      <c r="D46" s="92"/>
-      <c r="E46" s="59"/>
-      <c r="F46" s="90"/>
-      <c r="G46" s="88"/>
+      <c r="B46" s="64"/>
+      <c r="C46" s="59" t="s">
+        <v>65</v>
+      </c>
+      <c r="D46" s="67"/>
+      <c r="E46" s="79"/>
+      <c r="F46" s="55"/>
+      <c r="G46" s="92"/>
       <c r="H46" s="6"/>
     </row>
     <row r="47" spans="1:11" ht="39" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B47" s="110"/>
-      <c r="C47" s="61"/>
-      <c r="D47" s="93"/>
-      <c r="E47" s="60"/>
-      <c r="F47" s="90"/>
-      <c r="G47" s="88"/>
+      <c r="B47" s="65"/>
+      <c r="C47" s="59"/>
+      <c r="D47" s="68"/>
+      <c r="E47" s="80"/>
+      <c r="F47" s="55"/>
+      <c r="G47" s="92"/>
       <c r="H47" s="4"/>
     </row>
     <row r="48" spans="1:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B48" s="58" t="s">
-        <v>35</v>
-      </c>
-      <c r="C48" s="58" t="s">
-        <v>63</v>
-      </c>
-      <c r="D48" s="91" t="s">
-        <v>58</v>
-      </c>
-      <c r="E48" s="58" t="s">
-        <v>44</v>
-      </c>
-      <c r="F48" s="48"/>
-      <c r="G48" s="88"/>
+      <c r="B48" s="78" t="s">
+        <v>34</v>
+      </c>
+      <c r="C48" s="78" t="s">
+        <v>62</v>
+      </c>
+      <c r="D48" s="66" t="s">
+        <v>57</v>
+      </c>
+      <c r="E48" s="78" t="s">
+        <v>43</v>
+      </c>
+      <c r="F48" s="45"/>
+      <c r="G48" s="92"/>
     </row>
     <row r="49" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="B49" s="59"/>
-      <c r="C49" s="59"/>
-      <c r="D49" s="92"/>
-      <c r="E49" s="59"/>
-      <c r="F49" s="90" t="s">
-        <v>41</v>
-      </c>
-      <c r="G49" s="88"/>
+      <c r="B49" s="79"/>
+      <c r="C49" s="79"/>
+      <c r="D49" s="67"/>
+      <c r="E49" s="79"/>
+      <c r="F49" s="55" t="s">
+        <v>40</v>
+      </c>
+      <c r="G49" s="92"/>
     </row>
     <row r="50" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B50" s="60"/>
-      <c r="C50" s="60"/>
-      <c r="D50" s="93"/>
-      <c r="E50" s="60"/>
-      <c r="F50" s="90"/>
-      <c r="G50" s="88"/>
+      <c r="B50" s="80"/>
+      <c r="C50" s="80"/>
+      <c r="D50" s="68"/>
+      <c r="E50" s="80"/>
+      <c r="F50" s="55"/>
+      <c r="G50" s="92"/>
     </row>
     <row r="51" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="B51" s="38"/>
-      <c r="C51" s="27"/>
-      <c r="D51" s="43"/>
-      <c r="E51" s="27"/>
-      <c r="F51" s="90"/>
-      <c r="G51" s="89"/>
+      <c r="B51" s="36"/>
+      <c r="C51" s="26"/>
+      <c r="D51" s="40"/>
+      <c r="E51" s="26"/>
+      <c r="F51" s="55"/>
+      <c r="G51" s="93"/>
     </row>
     <row r="52" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="B52" s="31"/>
-      <c r="C52" s="27"/>
-      <c r="D52" s="31"/>
-      <c r="E52" s="31"/>
-      <c r="F52" s="31"/>
+        <v>49</v>
+      </c>
+      <c r="B52" s="30"/>
+      <c r="C52" s="26"/>
+      <c r="D52" s="30"/>
+      <c r="E52" s="30"/>
+      <c r="F52" s="30"/>
       <c r="G52" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="84">
+    <mergeCell ref="K32:K33"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="E33:E35"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="H32:H33"/>
+    <mergeCell ref="I20:I21"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="I18:I19"/>
+    <mergeCell ref="G13:G51"/>
+    <mergeCell ref="F49:F51"/>
+    <mergeCell ref="D48:D50"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="D42:D44"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="F36:F37"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="E48:E50"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C48:C50"/>
+    <mergeCell ref="B48:B50"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="E45:E47"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="C36:C38"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B10:B11"/>
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="B14:B15"/>
@@ -2029,79 +2079,11 @@
     <mergeCell ref="B33:B34"/>
     <mergeCell ref="D33:D34"/>
     <mergeCell ref="B37:B38"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="E45:E47"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="C36:C38"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="E48:E50"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C48:C50"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="H32:H33"/>
-    <mergeCell ref="I20:I21"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="I18:I19"/>
-    <mergeCell ref="G13:G51"/>
-    <mergeCell ref="F49:F51"/>
-    <mergeCell ref="D48:D50"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="D42:D44"/>
-    <mergeCell ref="K32:K33"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E26:E27"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="F26:F27"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F36:F37"/>
-    <mergeCell ref="E33:E35"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="B48:B50"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="C31:C33"/>
-    <mergeCell ref="C25:C26"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.74803149606299213" right="0.55118110236220474" top="0.78740157480314965" bottom="0.78740157480314965" header="0.51181102362204722" footer="0.51181102362204722"/>
-  <pageSetup scale="37" firstPageNumber="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="300"/>
+  <pageSetup scale="38" firstPageNumber="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="300"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
</xml_diff>